<commit_message>
Update trial member data by removing specific identifier
Update the title of the trial member data file to reflect recent changes and remove the word "الأسد" from the member data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 8172dddf-91c5-4b07-b0fd-6b00377b3241
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 02239335-5f8a-4a23-aeda-6dbe490cef7a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/32befe2c-e84a-43de-b1ea-e62eeeff820d/8172dddf-91c5-4b07-b0fd-6b00377b3241/HDfQU52
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/اعضاء-تجريبيون-SCVA.xlsx
+++ b/اعضاء-تجريبيون-SCVA.xlsx
@@ -398,23 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O101"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="28.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="32.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2049,7 +2032,7 @@
         <v>السويداء</v>
       </c>
       <c r="L35" t="str">
-        <v>مستشفى الأسد الجامعي - السويداء</v>
+        <v>مستشفى الجمهوري الجامعي - السويداء</v>
       </c>
       <c r="M35" t="str">
         <v>2007-10-01</v>
@@ -2096,7 +2079,7 @@
         <v>درعا</v>
       </c>
       <c r="L36" t="str">
-        <v>مستشفى الأسد الجامعي - درعا</v>
+        <v>مستشفى الجمهوري الجامعي - درعا</v>
       </c>
       <c r="M36" t="str">
         <v>2004-12-01</v>

</xml_diff>